<commit_message>
Add Invoice Template and Finance Template to Module 3
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pdfs/sg-finance-template.xlsx
+++ b/pdfs/sg-finance-template.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessh\Downloads\Claude-Setup\lms\solid-ground\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D36E513-3E49-4B9D-83FF-126BBD7A04D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601FA871-3063-4979-BE04-B4293BD60002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="1" r:id="rId1"/>
     <sheet name="Household Budget" sheetId="2" r:id="rId2"/>
     <sheet name="Shared Expenses" sheetId="3" r:id="rId3"/>
-    <sheet name="Sales Forecast" sheetId="4" r:id="rId4"/>
-    <sheet name="Marketing Plan" sheetId="5" r:id="rId5"/>
-    <sheet name="Cash Flow Budget" sheetId="6" r:id="rId6"/>
-    <sheet name="Profit &amp; Loss" sheetId="7" r:id="rId7"/>
-    <sheet name="Dashboard" sheetId="8" r:id="rId8"/>
+    <sheet name="Service Pricing" sheetId="4" r:id="rId4"/>
+    <sheet name="Sales Forecast" sheetId="5" r:id="rId5"/>
+    <sheet name="Marketing Plan" sheetId="6" r:id="rId6"/>
+    <sheet name="Cash Flow Budget" sheetId="7" r:id="rId7"/>
+    <sheet name="Profit &amp; Loss" sheetId="8" r:id="rId8"/>
+    <sheet name="Dashboard" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,118 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="247">
+  <si>
+    <t>PROFIT &amp; LOSS STATEMENT - Year 1</t>
+  </si>
+  <si>
+    <t>INCOME</t>
+  </si>
+  <si>
+    <t>Total Sales</t>
+  </si>
+  <si>
+    <t>Less: GST collected (if registered)</t>
+  </si>
+  <si>
+    <t>Net Sales (excl. GST)</t>
+  </si>
+  <si>
+    <t>Less: Variable costs</t>
+  </si>
+  <si>
+    <t>CONTRIBUTION MARGIN</t>
+  </si>
+  <si>
+    <t>OVERHEAD EXPENSES</t>
+  </si>
+  <si>
+    <t>Accountant / bookkeeper</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Electricity / gas</t>
+  </si>
+  <si>
+    <t>Postage / courier</t>
+  </si>
+  <si>
+    <t>Rent (studio / clinic / market stall)</t>
+  </si>
+  <si>
+    <t>Licenses &amp; permits</t>
+  </si>
+  <si>
+    <t>Insurance - professional indemnity</t>
+  </si>
+  <si>
+    <t>Insurance - public liability</t>
+  </si>
+  <si>
+    <t>Phone / internet / mobile (business %)</t>
+  </si>
+  <si>
+    <t>Fuel (business %)</t>
+  </si>
+  <si>
+    <t>Vehicle costs (business %)</t>
+  </si>
+  <si>
+    <t>Bank charges</t>
+  </si>
+  <si>
+    <t>Subscriptions / software</t>
+  </si>
+  <si>
+    <t>Professional development / training</t>
+  </si>
+  <si>
+    <t>Spare 1</t>
+  </si>
+  <si>
+    <t>Spare 2</t>
+  </si>
+  <si>
+    <t>Spare 3</t>
+  </si>
+  <si>
+    <t>(spare 4)</t>
+  </si>
+  <si>
+    <t>Personal super contributions</t>
+  </si>
+  <si>
+    <t>Total Overhead Expenses</t>
+  </si>
+  <si>
+    <t>NET PROFIT BEFORE DRAWINGS</t>
+  </si>
+  <si>
+    <t>Less: Drawings</t>
+  </si>
+  <si>
+    <t>NET PROFIT BEFORE TAX</t>
+  </si>
+  <si>
+    <t>TAX CALCULATION (2024-25 ATO Rates - Sole Trader)</t>
+  </si>
+  <si>
+    <t>Taxable income</t>
+  </si>
+  <si>
+    <t>Estimated income tax</t>
+  </si>
+  <si>
+    <t>Medicare Levy (2%)</t>
+  </si>
+  <si>
+    <t>Total tax payable</t>
+  </si>
+  <si>
+    <t>NET PROFIT AFTER TAX</t>
+  </si>
   <si>
     <t>SOLID GROUND - Business Setup</t>
   </si>
@@ -150,9 +262,6 @@
     <t>Annual Total</t>
   </si>
   <si>
-    <t>INCOME</t>
-  </si>
-  <si>
     <t>Casual/Part-time wages</t>
   </si>
   <si>
@@ -309,12 +418,6 @@
     <t>Home office (utilities portion)</t>
   </si>
   <si>
-    <t>Spare 1</t>
-  </si>
-  <si>
-    <t>Spare 2</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
@@ -345,6 +448,87 @@
     <t>Spare</t>
   </si>
   <si>
+    <t>Service Pricing Calculator</t>
+  </si>
+  <si>
+    <t>Module 6 - Solid Ground  |  Fill in the yellow cells</t>
+  </si>
+  <si>
+    <t>STEP 1 — Your weekly expenses</t>
+  </si>
+  <si>
+    <t>Weekly business expenses</t>
+  </si>
+  <si>
+    <t>Rent, insurance, software, subscriptions, supplies</t>
+  </si>
+  <si>
+    <t>Weekly personal expenses</t>
+  </si>
+  <si>
+    <t>Rent/mortgage, groceries, bills - what you need to live on</t>
+  </si>
+  <si>
+    <t>Business expenses target (first goal)</t>
+  </si>
+  <si>
+    <t>Full income target (business + personal)</t>
+  </si>
+  <si>
+    <t>STEP 2 — Your hourly rate</t>
+  </si>
+  <si>
+    <t>My hourly rate (current or considering)</t>
+  </si>
+  <si>
+    <t>What you charge per hour or per session</t>
+  </si>
+  <si>
+    <t>STEP 3 — Realistic client hours per week</t>
+  </si>
+  <si>
+    <t>Hours I CAN see clients</t>
+  </si>
+  <si>
+    <t>Max available hours</t>
+  </si>
+  <si>
+    <t>Hours I WANT to see clients</t>
+  </si>
+  <si>
+    <t>What feels right and sustainable</t>
+  </si>
+  <si>
+    <t>STEP 4 — What your rate earns you</t>
+  </si>
+  <si>
+    <t>Income at your rate x hours you CAN work</t>
+  </si>
+  <si>
+    <t>Income at your rate x hours you WANT to work</t>
+  </si>
+  <si>
+    <t>Hours needed to cover business expenses (at your rate)</t>
+  </si>
+  <si>
+    <t>Hours needed to cover full expenses (at your rate)</t>
+  </si>
+  <si>
+    <t>STEP 5 — Gap check</t>
+  </si>
+  <si>
+    <t>Does your rate cover business expenses at WANT hours?</t>
+  </si>
+  <si>
+    <t>Rate needed to cover business expenses at WANT hours</t>
+  </si>
+  <si>
+    <t>Rate needed to cover FULL expenses at WANT hours</t>
+  </si>
+  <si>
+    <t>Your starting price is not your forever price. Begin with a number you can say without flinching. Revisit after 6-12 months.</t>
+  </si>
+  <si>
     <t>SALES FORECAST</t>
   </si>
   <si>
@@ -525,63 +709,12 @@
     <t>GST on variable costs (only if GST registered)</t>
   </si>
   <si>
-    <t>CONTRIBUTION MARGIN</t>
-  </si>
-  <si>
     <t>What is a contribution margin? Sales minus the direct costs of making those sales.</t>
   </si>
   <si>
     <t>OVERHEAD EXPENSES OUT</t>
   </si>
   <si>
-    <t>Accountant / bookkeeper</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Electricity / gas</t>
-  </si>
-  <si>
-    <t>Postage / courier</t>
-  </si>
-  <si>
-    <t>Rent (studio / clinic / market stall)</t>
-  </si>
-  <si>
-    <t>Licenses &amp; permits</t>
-  </si>
-  <si>
-    <t>Insurance - professional indemnity</t>
-  </si>
-  <si>
-    <t>Insurance - public liability</t>
-  </si>
-  <si>
-    <t>Phone / internet / mobile (business %)</t>
-  </si>
-  <si>
-    <t>Fuel (business %)</t>
-  </si>
-  <si>
-    <t>Vehicle costs (business %)</t>
-  </si>
-  <si>
-    <t>Bank charges</t>
-  </si>
-  <si>
-    <t>Subscriptions / software</t>
-  </si>
-  <si>
-    <t>Professional development / training</t>
-  </si>
-  <si>
-    <t>Spare 3</t>
-  </si>
-  <si>
-    <t>(spare 4)</t>
-  </si>
-  <si>
     <t>Personal super contributions (voluntary)</t>
   </si>
   <si>
@@ -604,57 +737,6 @@
   </si>
   <si>
     <t>Closing bank balance</t>
-  </si>
-  <si>
-    <t>PROFIT &amp; LOSS STATEMENT - Year 1</t>
-  </si>
-  <si>
-    <t>Total Sales</t>
-  </si>
-  <si>
-    <t>Less: GST collected (if registered)</t>
-  </si>
-  <si>
-    <t>Net Sales (excl. GST)</t>
-  </si>
-  <si>
-    <t>Less: Variable costs</t>
-  </si>
-  <si>
-    <t>OVERHEAD EXPENSES</t>
-  </si>
-  <si>
-    <t>Personal super contributions</t>
-  </si>
-  <si>
-    <t>Total Overhead Expenses</t>
-  </si>
-  <si>
-    <t>NET PROFIT BEFORE DRAWINGS</t>
-  </si>
-  <si>
-    <t>Less: Drawings</t>
-  </si>
-  <si>
-    <t>NET PROFIT BEFORE TAX</t>
-  </si>
-  <si>
-    <t>TAX CALCULATION (2024-25 ATO Rates - Sole Trader)</t>
-  </si>
-  <si>
-    <t>Taxable income</t>
-  </si>
-  <si>
-    <t>Estimated income tax</t>
-  </si>
-  <si>
-    <t>Medicare Levy (2%)</t>
-  </si>
-  <si>
-    <t>Total tax payable</t>
-  </si>
-  <si>
-    <t>NET PROFIT AFTER TAX</t>
   </si>
   <si>
     <t>SOLID GROUND - Financial Dashboard</t>
@@ -706,12 +788,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;\(\$#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot; hrs/wk&quot;"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -803,8 +888,71 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFD0D9DC"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E2E32"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1E2E32"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF888888"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF1E2E32"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3B5E6E"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1E2E32"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF065F46"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -831,8 +979,33 @@
         <fgColor rgb="FFE4EAEC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E2E32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A7080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAF7F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8E0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -840,11 +1013,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999900"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999900"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999900"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999900"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -944,15 +1132,59 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="20" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -962,9 +1194,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1277,97 +1506,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="3" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
+      <c r="A3" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
     </row>
     <row r="5" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="3" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="3" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B9" s="32"/>
       <c r="C9" s="33" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B11" s="5">
         <v>0.1</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="B12" s="6">
         <v>18200</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1384,7 +1613,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -1393,112 +1622,112 @@
   <dimension ref="A1:N44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="38.109375" customWidth="1"/>
     <col min="2" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
     </row>
     <row r="2" spans="1:14" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
+      <c r="A2" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
     </row>
     <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
+      <c r="A5" s="46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -1519,7 +1748,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1540,7 +1769,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1561,7 +1790,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1582,7 +1811,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1603,7 +1832,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="B11" s="11">
         <f t="shared" ref="B11:N11" si="0">SUM(B6:B10)</f>
@@ -1659,31 +1888,31 @@
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="36"/>
-      <c r="K13" s="36"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="36"/>
-      <c r="N13" s="36"/>
+      <c r="A13" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="45"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1704,7 +1933,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1725,7 +1954,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1746,7 +1975,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1767,7 +1996,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1788,7 +2017,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1809,12 +2038,12 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1835,7 +2064,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1856,7 +2085,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1877,7 +2106,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1898,7 +2127,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1919,17 +2148,17 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1950,7 +2179,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1971,7 +2200,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1992,12 +2221,12 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -2018,7 +2247,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -2039,12 +2268,12 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -2065,7 +2294,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2086,7 +2315,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -2107,7 +2336,7 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -2128,7 +2357,7 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -2149,7 +2378,7 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="B41" s="11">
         <f t="shared" ref="B41:N41" si="2">SUM(B14:B39)</f>
@@ -2206,7 +2435,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="B42" s="11">
         <f t="shared" ref="B42:N42" si="3">B11-B40</f>
@@ -2263,7 +2492,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="B43" s="6">
         <v>0</v>
@@ -2282,7 +2511,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="B44" s="9">
         <f>B42+B41</f>
@@ -2360,58 +2589,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="A2" s="49" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
+      <c r="A4" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="B6" s="6">
         <v>0</v>
@@ -2434,7 +2663,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="B7" s="6">
         <v>0</v>
@@ -2457,7 +2686,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="B8" s="6">
         <v>0</v>
@@ -2480,7 +2709,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="B9" s="6">
         <v>0</v>
@@ -2503,7 +2732,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="B10" s="6">
         <v>0</v>
@@ -2526,7 +2755,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="B11" s="6">
         <v>0</v>
@@ -2549,7 +2778,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
       <c r="B12" s="6">
         <v>0</v>
@@ -2572,7 +2801,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="B13" s="6">
         <v>0</v>
@@ -2595,7 +2824,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="B14" s="6">
         <v>0</v>
@@ -2618,7 +2847,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="B15" s="11">
         <f>SUM(B6:B14)</f>
@@ -2634,38 +2863,38 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="37" t="s">
-        <v>92</v>
-      </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
+      <c r="A17" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
       <c r="B19" s="6">
         <v>0</v>
@@ -2688,7 +2917,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>97</v>
+        <v>131</v>
       </c>
       <c r="B20" s="6">
         <v>0</v>
@@ -2711,7 +2940,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>98</v>
+        <v>132</v>
       </c>
       <c r="B21" s="6">
         <v>0</v>
@@ -2734,7 +2963,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -2757,7 +2986,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>99</v>
+        <v>133</v>
       </c>
       <c r="B23" s="6">
         <v>0</v>
@@ -2780,7 +3009,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>100</v>
+        <v>134</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -2803,7 +3032,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="B25" s="11">
         <f>SUM(B19:B24)</f>
@@ -2820,9 +3049,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2831,6 +3060,291 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="50.33203125" customWidth="1"/>
+    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+    </row>
+    <row r="2" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="54" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+    </row>
+    <row r="3" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="35"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+    </row>
+    <row r="4" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+    </row>
+    <row r="5" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="52" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="45"/>
+    </row>
+    <row r="6" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="37"/>
+      <c r="C6" s="52" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="45"/>
+    </row>
+    <row r="7" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" s="39" t="str">
+        <f>IF(B5&gt;0,B5,"")</f>
+        <v/>
+      </c>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+    </row>
+    <row r="8" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="39" t="str">
+        <f>IF((B5+B6)&gt;0,B5+B6,"")</f>
+        <v/>
+      </c>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+    </row>
+    <row r="9" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+    </row>
+    <row r="10" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+    </row>
+    <row r="11" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" s="37"/>
+      <c r="C11" s="52" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11" s="45"/>
+    </row>
+    <row r="12" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+    </row>
+    <row r="13" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="51" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+    </row>
+    <row r="14" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14" s="41"/>
+      <c r="C14" s="52" t="s">
+        <v>149</v>
+      </c>
+      <c r="D14" s="45"/>
+    </row>
+    <row r="15" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" s="41"/>
+      <c r="C15" s="52" t="s">
+        <v>151</v>
+      </c>
+      <c r="D15" s="45"/>
+    </row>
+    <row r="16" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+    </row>
+    <row r="17" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+    </row>
+    <row r="18" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" s="42">
+        <f>IFERROR(B11*B14,"")</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+    </row>
+    <row r="19" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="38" t="s">
+        <v>154</v>
+      </c>
+      <c r="B19" s="42">
+        <f>IFERROR(B11*B15,"")</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+    </row>
+    <row r="20" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="35"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+    </row>
+    <row r="21" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="43" t="str">
+        <f>IFERROR(IF(B11&gt;0,B5/B11,""),"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+    </row>
+    <row r="22" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22" s="43" t="str">
+        <f>IFERROR(IF(B11&gt;0,(B5+B6)/B11,""),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+    </row>
+    <row r="23" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="35"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+    </row>
+    <row r="24" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+    </row>
+    <row r="25" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="B25" s="44" t="str">
+        <f>IFERROR(IF(B15*B11&gt;=B5,"Yes - covered","Gap - see below"),"")</f>
+        <v>Yes - covered</v>
+      </c>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+    </row>
+    <row r="26" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="B26" s="39" t="str">
+        <f>IFERROR(IF(B15&gt;0,B5/B15,""),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+    </row>
+    <row r="27" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="39" t="str">
+        <f>IFERROR(IF(B15&gt;0,(B5+B6)/B15,""),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+    </row>
+    <row r="28" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+    </row>
+    <row r="29" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="53" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" s="45"/>
+      <c r="C29" s="45"/>
+      <c r="D29" s="45"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C5:D5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2842,121 +3356,121 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
     </row>
     <row r="2" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
+      <c r="A2" s="49" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
+      <c r="A4" s="46" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="45"/>
+      <c r="O4" s="45"/>
+      <c r="P4" s="45"/>
+      <c r="Q4" s="45"/>
     </row>
     <row r="5" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>104</v>
+        <v>165</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>105</v>
+        <v>166</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="O5" s="18" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="P5" s="18" t="s">
-        <v>106</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
-        <v>107</v>
+        <v>168</v>
       </c>
       <c r="B6" s="6">
         <v>0</v>
@@ -3008,7 +3522,7 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="31" t="s">
-        <v>108</v>
+        <v>169</v>
       </c>
       <c r="B7" s="6">
         <v>0</v>
@@ -3060,7 +3574,7 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="31" t="s">
-        <v>109</v>
+        <v>170</v>
       </c>
       <c r="B8" s="6">
         <v>0</v>
@@ -3112,7 +3626,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="31" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="B9" s="6">
         <v>0</v>
@@ -3164,7 +3678,7 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="31" t="s">
-        <v>111</v>
+        <v>172</v>
       </c>
       <c r="B10" s="6">
         <v>0</v>
@@ -3216,7 +3730,7 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="31" t="s">
-        <v>112</v>
+        <v>173</v>
       </c>
       <c r="B11" s="6">
         <v>0</v>
@@ -3268,7 +3782,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="31" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="B12" s="6">
         <v>0</v>
@@ -3320,7 +3834,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="31" t="s">
-        <v>114</v>
+        <v>175</v>
       </c>
       <c r="B13" s="6">
         <v>0</v>
@@ -3372,7 +3886,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="31" t="s">
-        <v>115</v>
+        <v>176</v>
       </c>
       <c r="B14" s="6">
         <v>0</v>
@@ -3424,7 +3938,7 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="31" t="s">
-        <v>116</v>
+        <v>177</v>
       </c>
       <c r="B15" s="6">
         <v>0</v>
@@ -3475,10 +3989,10 @@
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A16" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="B16" s="36"/>
+      <c r="A16" s="55" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="45"/>
       <c r="C16" s="11">
         <f t="shared" ref="C16:N16" si="2">SUM(C6:C15)</f>
         <v>0</v>
@@ -3537,50 +4051,50 @@
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" s="37" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
+      <c r="A18" s="46" t="s">
+        <v>179</v>
+      </c>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="45"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="45"/>
+      <c r="O18" s="45"/>
+      <c r="P18" s="45"/>
+      <c r="Q18" s="45"/>
     </row>
     <row r="19" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="38" t="s">
-        <v>119</v>
-      </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="36"/>
-      <c r="O19" s="36"/>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="36"/>
+      <c r="A19" s="49" t="s">
+        <v>180</v>
+      </c>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="45"/>
+      <c r="M19" s="45"/>
+      <c r="N19" s="45"/>
+      <c r="O19" s="45"/>
+      <c r="P19" s="45"/>
+      <c r="Q19" s="45"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>120</v>
+        <v>181</v>
       </c>
       <c r="B20" s="5">
         <v>1</v>
@@ -3588,7 +4102,7 @@
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>121</v>
+        <v>182</v>
       </c>
       <c r="B21" s="5">
         <v>0</v>
@@ -3596,7 +4110,7 @@
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>122</v>
+        <v>183</v>
       </c>
       <c r="B22" s="5">
         <v>0</v>
@@ -3604,7 +4118,7 @@
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
-        <v>123</v>
+        <v>184</v>
       </c>
       <c r="B23" s="21">
         <f>B20+B21+B22</f>
@@ -3613,7 +4127,7 @@
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>124</v>
+        <v>185</v>
       </c>
       <c r="C24" s="9">
         <f>C16*$B$20</f>
@@ -3669,92 +4183,92 @@
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A26" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="36"/>
-      <c r="J26" s="36"/>
-      <c r="K26" s="36"/>
-      <c r="L26" s="36"/>
-      <c r="M26" s="36"/>
-      <c r="N26" s="36"/>
-      <c r="O26" s="36"/>
-      <c r="P26" s="36"/>
-      <c r="Q26" s="36"/>
+      <c r="A26" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="45"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="45"/>
+      <c r="L26" s="45"/>
+      <c r="M26" s="45"/>
+      <c r="N26" s="45"/>
+      <c r="O26" s="45"/>
+      <c r="P26" s="45"/>
+      <c r="Q26" s="45"/>
     </row>
     <row r="27" spans="1:17" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="36"/>
-      <c r="O27" s="36"/>
-      <c r="P27" s="36"/>
-      <c r="Q27" s="36"/>
+      <c r="A27" s="49" t="s">
+        <v>187</v>
+      </c>
+      <c r="B27" s="45"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="45"/>
+      <c r="J27" s="45"/>
+      <c r="K27" s="45"/>
+      <c r="L27" s="45"/>
+      <c r="M27" s="45"/>
+      <c r="N27" s="45"/>
+      <c r="O27" s="45"/>
+      <c r="P27" s="45"/>
+      <c r="Q27" s="45"/>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>104</v>
+        <v>165</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>127</v>
+        <v>188</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="L28" s="8" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="M28" s="8" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="N28" s="8" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="O28" s="8" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="P28" s="8"/>
     </row>
@@ -4369,10 +4883,10 @@
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="B39" s="36"/>
+      <c r="A39" s="55" t="s">
+        <v>189</v>
+      </c>
+      <c r="B39" s="45"/>
       <c r="C39" s="11">
         <f t="shared" ref="C39:N39" si="17">SUM(C29:C38)</f>
         <v>0</v>
@@ -4442,8 +4956,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:O26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4454,112 +4968,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
     </row>
     <row r="2" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
+      <c r="A2" s="49" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
+      <c r="A5" s="46" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>132</v>
+        <v>193</v>
       </c>
       <c r="B6" s="6">
         <v>0</v>
@@ -4607,7 +5121,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>133</v>
+        <v>194</v>
       </c>
       <c r="B7" s="6">
         <v>0</v>
@@ -4655,7 +5169,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>134</v>
+        <v>195</v>
       </c>
       <c r="B8" s="6">
         <v>0</v>
@@ -4703,7 +5217,7 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>135</v>
+        <v>196</v>
       </c>
       <c r="B9" s="6">
         <v>0</v>
@@ -4750,27 +5264,27 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="37" t="s">
-        <v>136</v>
-      </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="36"/>
+      <c r="A10" s="46" t="s">
+        <v>197</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="45"/>
+      <c r="O10" s="45"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>137</v>
+        <v>198</v>
       </c>
       <c r="B11" s="6">
         <v>0</v>
@@ -4818,7 +5332,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>138</v>
+        <v>199</v>
       </c>
       <c r="B12" s="6">
         <v>0</v>
@@ -4866,7 +5380,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>139</v>
+        <v>200</v>
       </c>
       <c r="B13" s="6">
         <v>0</v>
@@ -4914,7 +5428,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>140</v>
+        <v>201</v>
       </c>
       <c r="B14" s="6">
         <v>0</v>
@@ -4961,27 +5475,27 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
-      <c r="N15" s="36"/>
-      <c r="O15" s="36"/>
+      <c r="A15" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>142</v>
+        <v>203</v>
       </c>
       <c r="B16" s="6">
         <v>0</v>
@@ -5029,7 +5543,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>143</v>
+        <v>204</v>
       </c>
       <c r="B17" s="6">
         <v>0</v>
@@ -5077,7 +5591,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="B18" s="6">
         <v>0</v>
@@ -5124,27 +5638,27 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="36"/>
-      <c r="O19" s="36"/>
+      <c r="A19" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="45"/>
+      <c r="M19" s="45"/>
+      <c r="N19" s="45"/>
+      <c r="O19" s="45"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>146</v>
+        <v>207</v>
       </c>
       <c r="B20" s="6">
         <v>0</v>
@@ -5192,7 +5706,7 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>147</v>
+        <v>208</v>
       </c>
       <c r="B21" s="6">
         <v>0</v>
@@ -5240,7 +5754,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>148</v>
+        <v>209</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -5288,7 +5802,7 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="B23" s="6">
         <v>0</v>
@@ -5336,7 +5850,7 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -5384,7 +5898,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="B25" s="6">
         <v>0</v>
@@ -5431,10 +5945,10 @@
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="B26" s="36"/>
+      <c r="A26" s="55" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" s="45"/>
       <c r="C26" s="11">
         <f t="shared" ref="C26:O26" si="1">SUM(C6:C25)</f>
         <v>0</v>
@@ -5502,8 +6016,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5513,88 +6027,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>152</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
+      <c r="A4" s="46" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+      <c r="N4" s="45"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>153</v>
+        <v>214</v>
       </c>
       <c r="B5" s="9">
         <f>'Sales Forecast'!B24</f>
@@ -5651,7 +6165,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>154</v>
+        <v>215</v>
       </c>
       <c r="B6" s="6">
         <v>0</v>
@@ -5696,7 +6210,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>155</v>
+        <v>216</v>
       </c>
       <c r="B7" s="6">
         <v>0</v>
@@ -5741,7 +6255,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>156</v>
+        <v>217</v>
       </c>
       <c r="B8" s="9">
         <f>IF(Setup!$B$9="Yes",B5/11,0)</f>
@@ -5798,7 +6312,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>157</v>
+        <v>218</v>
       </c>
       <c r="B9" s="11">
         <f t="shared" ref="B9:M9" si="0">B5+B6+B7</f>
@@ -5854,26 +6368,26 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="36"/>
-      <c r="N11" s="36"/>
+      <c r="A11" s="46" t="s">
+        <v>219</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>159</v>
+        <v>220</v>
       </c>
       <c r="B12" s="9">
         <f>'Sales Forecast'!B39</f>
@@ -5930,7 +6444,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>160</v>
+        <v>221</v>
       </c>
       <c r="B13" s="9">
         <f>IF(Setup!$B$9="Yes",B12/11,0)</f>
@@ -5987,7 +6501,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
       <c r="B14" s="24">
         <f t="shared" ref="B14:N14" si="1">B5-B12</f>
@@ -6043,44 +6557,44 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
-      <c r="N15" s="36"/>
+      <c r="A15" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="37" t="s">
-        <v>163</v>
-      </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
+      <c r="A17" s="46" t="s">
+        <v>223</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>164</v>
+        <v>8</v>
       </c>
       <c r="B18" s="6">
         <v>0</v>
@@ -6125,7 +6639,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>165</v>
+        <v>9</v>
       </c>
       <c r="B19" s="9">
         <f>'Marketing Plan'!B26</f>
@@ -6182,7 +6696,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>166</v>
+        <v>10</v>
       </c>
       <c r="B20" s="6">
         <v>0</v>
@@ -6227,7 +6741,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>167</v>
+        <v>11</v>
       </c>
       <c r="B21" s="6">
         <v>0</v>
@@ -6272,7 +6786,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>168</v>
+        <v>12</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -6317,7 +6831,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>169</v>
+        <v>13</v>
       </c>
       <c r="B23" s="6">
         <v>0</v>
@@ -6362,7 +6876,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>170</v>
+        <v>14</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -6407,7 +6921,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>171</v>
+        <v>15</v>
       </c>
       <c r="B25" s="6">
         <v>0</v>
@@ -6452,7 +6966,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>172</v>
+        <v>16</v>
       </c>
       <c r="B26" s="6">
         <v>0</v>
@@ -6497,7 +7011,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>173</v>
+        <v>17</v>
       </c>
       <c r="B27" s="6">
         <v>0</v>
@@ -6542,7 +7056,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>174</v>
+        <v>18</v>
       </c>
       <c r="B28" s="6">
         <v>0</v>
@@ -6587,7 +7101,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>175</v>
+        <v>19</v>
       </c>
       <c r="B29" s="6">
         <v>0</v>
@@ -6632,7 +7146,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>176</v>
+        <v>20</v>
       </c>
       <c r="B30" s="6">
         <v>0</v>
@@ -6677,7 +7191,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>177</v>
+        <v>21</v>
       </c>
       <c r="B31" s="6">
         <v>0</v>
@@ -6722,7 +7236,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="B32" s="6">
         <v>0</v>
@@ -6767,7 +7281,7 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="B33" s="6">
         <v>0</v>
@@ -6812,7 +7326,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>178</v>
+        <v>24</v>
       </c>
       <c r="B34" s="6">
         <v>0</v>
@@ -6857,7 +7371,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>179</v>
+        <v>25</v>
       </c>
       <c r="B35" s="6">
         <v>0</v>
@@ -6902,7 +7416,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>180</v>
+        <v>224</v>
       </c>
       <c r="B36" s="6">
         <v>0</v>
@@ -6947,7 +7461,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>181</v>
+        <v>225</v>
       </c>
       <c r="B37" s="6">
         <v>0</v>
@@ -6992,7 +7506,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="10" t="s">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="B38" s="11">
         <f t="shared" ref="B38:N38" si="3">SUM(B18:B37)</f>
@@ -7048,26 +7562,26 @@
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="37" t="s">
-        <v>183</v>
-      </c>
-      <c r="B40" s="36"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="36"/>
-      <c r="F40" s="36"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="36"/>
-      <c r="I40" s="36"/>
-      <c r="J40" s="36"/>
-      <c r="K40" s="36"/>
-      <c r="L40" s="36"/>
-      <c r="M40" s="36"/>
-      <c r="N40" s="36"/>
+      <c r="A40" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="B40" s="45"/>
+      <c r="C40" s="45"/>
+      <c r="D40" s="45"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="45"/>
+      <c r="G40" s="45"/>
+      <c r="H40" s="45"/>
+      <c r="I40" s="45"/>
+      <c r="J40" s="45"/>
+      <c r="K40" s="45"/>
+      <c r="L40" s="45"/>
+      <c r="M40" s="45"/>
+      <c r="N40" s="45"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
-        <v>184</v>
+        <v>228</v>
       </c>
       <c r="B41" s="11">
         <f t="shared" ref="B41:N41" si="4">B12+B38</f>
@@ -7124,7 +7638,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>185</v>
+        <v>229</v>
       </c>
       <c r="B42" s="11">
         <f t="shared" ref="B42:N42" si="5">B9-B41</f>
@@ -7181,7 +7695,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
       <c r="B43" s="9">
         <f t="shared" ref="B43:N43" si="6">B8-B13</f>
@@ -7238,7 +7752,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="B44" s="6">
         <v>0</v>
@@ -7257,7 +7771,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="s">
-        <v>187</v>
+        <v>231</v>
       </c>
       <c r="B45" s="9">
         <f>B44+B42</f>
@@ -7325,8 +7839,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7335,20 +7849,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>188</v>
-      </c>
-      <c r="B1" s="36"/>
+      <c r="A1" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="36"/>
+      <c r="A3" s="46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="45"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>189</v>
+        <v>2</v>
       </c>
       <c r="B4" s="9">
         <f>'Sales Forecast'!P16</f>
@@ -7357,7 +7871,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>190</v>
+        <v>3</v>
       </c>
       <c r="B5" s="9">
         <f>'Cash Flow Budget'!N8</f>
@@ -7366,7 +7880,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>191</v>
+        <v>4</v>
       </c>
       <c r="B6" s="11">
         <f>B4-B5</f>
@@ -7375,7 +7889,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>192</v>
+        <v>5</v>
       </c>
       <c r="B7" s="9">
         <f>'Sales Forecast'!P39</f>
@@ -7384,7 +7898,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
       <c r="B8" s="24">
         <f>B6-B7</f>
@@ -7392,14 +7906,14 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="37" t="s">
-        <v>193</v>
-      </c>
-      <c r="B10" s="36"/>
+      <c r="A10" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="45"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>164</v>
+        <v>8</v>
       </c>
       <c r="B11" s="9">
         <f>'Cash Flow Budget'!N18</f>
@@ -7408,7 +7922,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>165</v>
+        <v>9</v>
       </c>
       <c r="B12" s="9">
         <f>'Cash Flow Budget'!N19</f>
@@ -7417,7 +7931,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>166</v>
+        <v>10</v>
       </c>
       <c r="B13" s="9">
         <f>'Cash Flow Budget'!N20</f>
@@ -7426,7 +7940,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>167</v>
+        <v>11</v>
       </c>
       <c r="B14" s="9">
         <f>'Cash Flow Budget'!N21</f>
@@ -7435,7 +7949,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>168</v>
+        <v>12</v>
       </c>
       <c r="B15" s="9">
         <f>'Cash Flow Budget'!N22</f>
@@ -7444,7 +7958,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>169</v>
+        <v>13</v>
       </c>
       <c r="B16" s="9">
         <f>'Cash Flow Budget'!N23</f>
@@ -7453,7 +7967,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>170</v>
+        <v>14</v>
       </c>
       <c r="B17" s="9">
         <f>'Cash Flow Budget'!N24</f>
@@ -7462,7 +7976,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>171</v>
+        <v>15</v>
       </c>
       <c r="B18" s="9">
         <f>'Cash Flow Budget'!N25</f>
@@ -7471,7 +7985,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>172</v>
+        <v>16</v>
       </c>
       <c r="B19" s="9">
         <f>'Cash Flow Budget'!N26</f>
@@ -7480,7 +7994,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>173</v>
+        <v>17</v>
       </c>
       <c r="B20" s="9">
         <f>'Cash Flow Budget'!N27</f>
@@ -7489,7 +8003,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>174</v>
+        <v>18</v>
       </c>
       <c r="B21" s="9">
         <f>'Cash Flow Budget'!N28</f>
@@ -7498,7 +8012,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>175</v>
+        <v>19</v>
       </c>
       <c r="B22" s="9">
         <f>'Cash Flow Budget'!N29</f>
@@ -7507,7 +8021,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>176</v>
+        <v>20</v>
       </c>
       <c r="B23" s="9">
         <f>'Cash Flow Budget'!N30</f>
@@ -7516,7 +8030,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>177</v>
+        <v>21</v>
       </c>
       <c r="B24" s="9">
         <f>'Cash Flow Budget'!N31</f>
@@ -7525,7 +8039,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="B25" s="9">
         <f>'Cash Flow Budget'!N32</f>
@@ -7534,7 +8048,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="B26" s="9">
         <f>'Cash Flow Budget'!N33</f>
@@ -7543,7 +8057,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>178</v>
+        <v>24</v>
       </c>
       <c r="B27" s="9">
         <f>'Cash Flow Budget'!N34</f>
@@ -7552,7 +8066,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>179</v>
+        <v>25</v>
       </c>
       <c r="B28" s="9">
         <f>'Cash Flow Budget'!N35</f>
@@ -7561,7 +8075,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>194</v>
+        <v>26</v>
       </c>
       <c r="B29" s="9">
         <f>'Cash Flow Budget'!N36</f>
@@ -7570,7 +8084,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>195</v>
+        <v>27</v>
       </c>
       <c r="B30" s="11">
         <f>SUM(B11:B29)</f>
@@ -7579,7 +8093,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
-        <v>196</v>
+        <v>28</v>
       </c>
       <c r="B31" s="11">
         <f>B8-B30</f>
@@ -7588,7 +8102,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>197</v>
+        <v>29</v>
       </c>
       <c r="B32" s="9">
         <f>'Cash Flow Budget'!N37</f>
@@ -7597,7 +8111,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="25" t="s">
-        <v>198</v>
+        <v>30</v>
       </c>
       <c r="B33" s="24">
         <f>B31-B32</f>
@@ -7605,14 +8119,14 @@
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="37" t="s">
-        <v>199</v>
-      </c>
-      <c r="B35" s="36"/>
+      <c r="A35" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="45"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>200</v>
+        <v>32</v>
       </c>
       <c r="B36" s="9">
         <f>MAX(0,B33)</f>
@@ -7621,7 +8135,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>201</v>
+        <v>33</v>
       </c>
       <c r="B37" s="9">
         <f>IF(B36&lt;=0,0,IF(B36&lt;=18200,0,IF(B36&lt;=45500,(B36-18200)*0.19,IF(B36&lt;=120000,5092+(B36-45500)*0.325,IF(B36&lt;=180000,29467+(B36-120000)*0.37,51667+(B36-180000)*0.45)))))</f>
@@ -7630,7 +8144,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>202</v>
+        <v>34</v>
       </c>
       <c r="B38" s="9">
         <f>IF(B36&gt;26000,B36*0.02,0)</f>
@@ -7639,7 +8153,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="10" t="s">
-        <v>203</v>
+        <v>35</v>
       </c>
       <c r="B39" s="11">
         <f>B37+B38</f>
@@ -7648,7 +8162,7 @@
     </row>
     <row r="40" spans="1:2" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="27" t="s">
-        <v>204</v>
+        <v>36</v>
       </c>
       <c r="B40" s="28">
         <f>B33-B39</f>
@@ -7656,8 +8170,8 @@
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="36"/>
-      <c r="B43" s="36"/>
+      <c r="A43" s="45"/>
+      <c r="B43" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7671,8 +8185,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7682,29 +8196,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="A1" s="56" t="s">
+        <v>232</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
     </row>
     <row r="2" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>206</v>
-      </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="A2" s="49" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>207</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="46" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="B5" s="29">
         <f>Setup!B5</f>
@@ -7713,7 +8227,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="B6" s="29">
         <f>Setup!B6</f>
@@ -7722,7 +8236,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="B7" s="29" t="str">
         <f>Setup!B8</f>
@@ -7731,7 +8245,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>208</v>
+        <v>235</v>
       </c>
       <c r="B8" s="30">
         <f>Setup!B7</f>
@@ -7740,7 +8254,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="B9" s="29">
         <f>Setup!B9</f>
@@ -7748,15 +8262,15 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="37" t="s">
-        <v>209</v>
-      </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="36"/>
+      <c r="A11" s="46" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>210</v>
+        <v>237</v>
       </c>
       <c r="B12" s="11">
         <f>'Sales Forecast'!P16</f>
@@ -7765,7 +8279,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>211</v>
+        <v>238</v>
       </c>
       <c r="B13" s="20">
         <f>IFERROR('Profit &amp; Loss'!B8/'Profit &amp; Loss'!B6,0)</f>
@@ -7774,7 +8288,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>212</v>
+        <v>239</v>
       </c>
       <c r="B14" s="11">
         <f>'Cash Flow Budget'!N38</f>
@@ -7783,7 +8297,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>213</v>
+        <v>240</v>
       </c>
       <c r="B15" s="11">
         <f>'Profit &amp; Loss'!B33</f>
@@ -7792,7 +8306,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>214</v>
+        <v>241</v>
       </c>
       <c r="B16" s="11">
         <f>'Profit &amp; Loss'!B40</f>
@@ -7801,7 +8315,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>215</v>
+        <v>242</v>
       </c>
       <c r="B17" s="11">
         <f>'Cash Flow Budget'!M45</f>
@@ -7817,15 +8331,15 @@
       <c r="B19" s="11"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="37" t="s">
-        <v>216</v>
-      </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
+      <c r="A21" s="46" t="s">
+        <v>243</v>
+      </c>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>217</v>
+        <v>244</v>
       </c>
       <c r="B22" s="11">
         <f>'Household Budget'!N11</f>
@@ -7834,7 +8348,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>218</v>
+        <v>245</v>
       </c>
       <c r="B23" s="11">
         <f>'Household Budget'!N40</f>
@@ -7843,7 +8357,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>219</v>
+        <v>246</v>
       </c>
       <c r="B24" s="11">
         <f>'Household Budget'!N11-'Household Budget'!N40</f>
@@ -7851,14 +8365,14 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="37"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36"/>
+      <c r="A26" s="46"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
     </row>
     <row r="27" spans="1:3" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="41"/>
-      <c r="C27" s="36"/>
+      <c r="B27" s="57"/>
+      <c r="C27" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>